<commit_message>
crear y actualizar presupuesto y usuario (empleado), crear proyecto funcional
</commit_message>
<xml_diff>
--- a/data/datos_reales/xlsx/DatosReales_CICES_Proyectos.xlsx
+++ b/data/datos_reales/xlsx/DatosReales_CICES_Proyectos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angie\IdeaProjects\cices-system\data\datos_reales\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53AD369-53C6-4203-99B4-0183B192A5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D83E387-E322-439B-B4EF-C4500A8E52EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7488" yWindow="384" windowWidth="14280" windowHeight="11856" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PROYECTO" sheetId="1" r:id="rId1"/>
@@ -1526,9 +1526,7 @@
       <c r="D7" s="5">
         <v>41</v>
       </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
+      <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
         <v>68</v>
       </c>
@@ -1718,9 +1716,7 @@
       <c r="D13" s="5">
         <v>41</v>
       </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
+      <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
         <v>68</v>
       </c>
@@ -1739,6 +1735,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>